<commit_message>
Site updated: 2022-07-04 07:47:41
</commit_message>
<xml_diff>
--- a/devops/keepalived/vrrp.xlsx
+++ b/devops/keepalived/vrrp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qcmoke\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\myblog\source\_posts\devops\keepalived\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7977B40-9D87-4539-907C-12B0860B0786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA20DFB-0210-4F33-854D-2794CD2A8E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{57D6825B-E365-4F0B-86B3-4EE0F29387C3}"/>
   </bookViews>
@@ -1135,11 +1135,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>563880</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:colOff>60960</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1055097" cy="283411"/>
+    <xdr:ext cx="1982915" cy="474489"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="82" name="文本框 81">
@@ -1153,8 +1153,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7269480" y="1082040"/>
-          <a:ext cx="1055097" cy="283411"/>
+          <a:off x="6766560" y="960120"/>
+          <a:ext cx="1982915" cy="474489"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1176,11 +1176,12 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
           <a:spAutoFit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
+          <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US" altLang="zh-CN" sz="1100" b="0" i="0">
               <a:solidFill>
@@ -1196,6 +1197,78 @@
           <a:r>
             <a:rPr lang="zh-CN" altLang="en-US" sz="1100"/>
             <a:t>心跳检测</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" altLang="zh-CN" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100"/>
+            <a:t>（</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="zh-CN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>选举</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>出的</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>MASTER</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>拥有</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>VIP</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100"/>
+            <a:t>）</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>

</xml_diff>